<commit_message>
Test report and demo user guide fix
 - Test report & traceability were not latest due to sync issues
   from Foqus
 - Also updated user guide to add details about VLAB path setting
   as existing doesn't work.

Signed-off-by: Prasad Jondhale <prasad.jondhale@ti.com>
</commit_message>
<xml_diff>
--- a/docs/test_report/ethfw_traceability.xlsx
+++ b/docs/test_report/ethfw_traceability.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr saveExternalLinkValues="0" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1005" yWindow="1005" windowWidth="15000" windowHeight="10005"/>
+    <workbookView xWindow="996" yWindow="996" windowWidth="15000" windowHeight="9996" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -155,9 +155,6 @@
     <t>Not satisfied (&lt;50% TC Passing)</t>
   </si>
   <si>
-    <t>4/2/2019</t>
-  </si>
-  <si>
     <t>ETHFW-162 : EthFW System Test - PMU Driver Integration</t>
   </si>
   <si>
@@ -176,6 +173,9 @@
     <t>IMPLEMENTED</t>
   </si>
   <si>
+    <t>4/3/2019</t>
+  </si>
+  <si>
     <t>0 %</t>
   </si>
   <si>
@@ -191,10 +191,10 @@
     <t>ETHFW-161 : EthFW System Test - GPTIMER Driver Integration</t>
   </si>
   <si>
+    <t>EthFw_J7_00.08.00_EA8</t>
+  </si>
+  <si>
     <t>Processor SDK Vision :EthFw Requirement to Test Traceability Report</t>
-  </si>
-  <si>
-    <t>EthFw_J7_00.08.00_EA8</t>
   </si>
 </sst>
 </file>
@@ -697,13 +697,13 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="B2:G23"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="35" style="1" customWidth="1"/>
     <col min="3" max="7" width="25" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="11" t="s">
         <v>14</v>
       </c>
@@ -713,9 +713,9 @@
       <c r="F2" s="10"/>
       <c r="G2" s="10"/>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12"/>
@@ -723,31 +723,31 @@
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
       <c r="G5" s="10"/>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>39</v>
       </c>
@@ -759,7 +759,7 @@
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>34</v>
       </c>
@@ -771,14 +771,14 @@
       <c r="F8" s="10"/>
       <c r="G8" s="10"/>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
         <v>44</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>7</v>
       </c>
@@ -789,7 +789,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>29</v>
       </c>
@@ -800,9 +800,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C14" s="4">
         <v>0</v>
@@ -811,7 +811,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
         <v>45</v>
       </c>
@@ -822,7 +822,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
         <v>40</v>
       </c>
@@ -833,7 +833,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
         <v>0</v>
       </c>
@@ -842,7 +842,7 @@
       </c>
       <c r="D17" s="3"/>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="9" t="s">
         <v>56</v>
       </c>
@@ -852,12 +852,12 @@
       <c r="F21" s="10"/>
       <c r="G21" s="10"/>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>54</v>
@@ -872,7 +872,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>19</v>
       </c>
@@ -903,7 +903,7 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultColWidth="15" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="15" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="25" style="1" customWidth="1"/>
     <col min="3" max="3" width="50" style="1" customWidth="1"/>
@@ -913,7 +913,7 @@
     <col min="8" max="8" width="12" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>6</v>
       </c>
@@ -924,7 +924,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>26</v>
@@ -933,13 +933,13 @@
         <v>25</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H1" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>9</v>
       </c>
@@ -954,7 +954,7 @@
         <v>5</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F2" s="16" t="s">
         <v>43</v>
@@ -966,7 +966,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>30</v>
       </c>
@@ -981,7 +981,7 @@
         <v>5</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F3" s="16" t="s">
         <v>43</v>
@@ -993,7 +993,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>30</v>
       </c>
@@ -1008,19 +1008,19 @@
         <v>5</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F4" s="16" t="s">
         <v>43</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H4" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>30</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F5" s="16" t="s">
         <v>43</v>
@@ -1047,7 +1047,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>30</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>5</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F6" s="16" t="s">
         <v>43</v>
@@ -1074,7 +1074,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>30</v>
       </c>
@@ -1089,7 +1089,7 @@
         <v>5</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F7" s="16" t="s">
         <v>43</v>
@@ -1101,7 +1101,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>30</v>
       </c>
@@ -1116,7 +1116,7 @@
         <v>5</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F8" s="16" t="s">
         <v>43</v>
@@ -1128,7 +1128,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>30</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>5</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F9" s="16" t="s">
         <v>43</v>
@@ -1155,7 +1155,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>30</v>
       </c>
@@ -1170,7 +1170,7 @@
         <v>5</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F10" s="16" t="s">
         <v>43</v>

</xml_diff>